<commit_message>
Update local changes in fa-grab-import-sap
</commit_message>
<xml_diff>
--- a/fa-grab-import-sap/SAP_Template import JE bằng WB.xlsx
+++ b/fa-grab-import-sap/SAP_Template import JE bằng WB.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thuy.ct\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thuan.pv\.vesper\skill-repos\itttg-Vesper-skills\fa-grab-import-sap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA25CDA3-F2CA-4ACC-AAE7-7B757CDF99F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14784367-E246-431B-A2E2-DA0E878C74DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" activeTab="1" xr2:uid="{8F1E7E9B-2F36-49AC-9B10-FF7336557F6B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8F1E7E9B-2F36-49AC-9B10-FF7336557F6B}"/>
   </bookViews>
   <sheets>
     <sheet name="JE-Header" sheetId="1" r:id="rId1"/>
     <sheet name="JE-Line" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'JE-Line'!$A$3:$W$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'JE-Line'!$A$3:$X$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="100">
   <si>
     <t>Nhập số thứ tự của phiếu</t>
   </si>
@@ -339,6 +339,9 @@
   </si>
   <si>
     <t>0106869738-005</t>
+  </si>
+  <si>
+    <t>Nhập ngày hóa đơn, format: YYYYMMDD</t>
   </si>
 </sst>
 </file>
@@ -426,7 +429,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -481,6 +484,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF59D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -510,7 +518,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -578,10 +586,14 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -898,21 +910,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B136DD02-A7D0-42B8-BBB1-92B703741EB9}">
   <dimension ref="A1:N7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="10.81640625" customWidth="1"/>
-    <col min="3" max="3" width="14.81640625" customWidth="1"/>
-    <col min="4" max="4" width="58.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" customWidth="1"/>
-    <col min="8" max="8" width="9.54296875" customWidth="1"/>
-    <col min="9" max="9" width="16.1796875" customWidth="1"/>
-    <col min="10" max="10" width="12.81640625" customWidth="1"/>
-    <col min="12" max="12" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" customWidth="1"/>
+    <col min="4" max="4" width="58.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" customWidth="1"/>
+    <col min="9" max="9" width="16.21875" customWidth="1"/>
+    <col min="10" max="10" width="12.77734375" customWidth="1"/>
+    <col min="12" max="12" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="10" customFormat="1" ht="76" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="10" customFormat="1" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -937,13 +949,13 @@
       <c r="J1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="43" t="s">
+      <c r="L1" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -974,11 +986,11 @@
       <c r="J2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -1009,11 +1021,11 @@
       <c r="J3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -1049,7 +1061,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -1085,7 +1097,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
@@ -1121,7 +1133,7 @@
         <v>10000000000</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>4</v>
       </c>
@@ -1168,33 +1180,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C1398C5-904C-49F7-9674-3AEBD223EAA3}">
-  <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AH246"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.54296875" style="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.81640625" style="42" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.54296875" style="42" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.90625"/>
-    <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.453125" style="20" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.1796875" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.1796875" style="16" customWidth="1"/>
-    <col min="12" max="12" width="15.90625" customWidth="1"/>
-    <col min="16" max="16" width="12.453125" customWidth="1"/>
-    <col min="17" max="19" width="8.81640625" style="24"/>
-    <col min="20" max="20" width="10.1796875" style="24" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.1796875" customWidth="1"/>
-    <col min="23" max="23" width="12.26953125" customWidth="1"/>
-    <col min="24" max="27" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="10" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="58.54296875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" style="42" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" style="42" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.44140625" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" style="16" customWidth="1"/>
+    <col min="12" max="12" width="15.88671875" customWidth="1"/>
+    <col min="14" max="14" width="11.77734375" customWidth="1"/>
+    <col min="17" max="17" width="12.44140625" customWidth="1"/>
+    <col min="18" max="20" width="8.77734375" style="24"/>
+    <col min="21" max="21" width="10.21875" style="24" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.21875" customWidth="1"/>
+    <col min="24" max="24" width="12.21875" customWidth="1"/>
+    <col min="25" max="28" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="58.5546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="8" customFormat="1" ht="88.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" s="8" customFormat="1" ht="93" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>21</v>
       </c>
@@ -1232,25 +1244,27 @@
       <c r="M1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9" t="s">
+      <c r="N1" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="Q1" s="21"/>
       <c r="R1" s="21"/>
       <c r="S1" s="21"/>
       <c r="T1" s="21"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9" t="s">
+      <c r="U1" s="21"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="X1" s="9"/>
       <c r="Y1" s="9"/>
       <c r="Z1" s="9"/>
       <c r="AA1" s="9"/>
@@ -1260,8 +1274,9 @@
       <c r="AE1" s="9"/>
       <c r="AF1" s="9"/>
       <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
     </row>
-    <row r="2" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>28</v>
       </c>
@@ -1301,68 +1316,71 @@
       <c r="M2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="Q2" s="22" t="s">
+      <c r="R2" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="R2" s="22" t="s">
+      <c r="S2" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="S2" s="22" t="s">
+      <c r="T2" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="T2" s="22" t="s">
+      <c r="U2" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="W2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="X2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="Y2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="Y2" s="2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="Z2" s="2" t="s">
+      <c r="AA2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AA2" s="2" t="s">
+      <c r="AB2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AC2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AC2" s="2" t="s">
+      <c r="AD2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AE2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AG2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1402,68 +1420,71 @@
       <c r="M3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="Q3" s="22" t="s">
+      <c r="R3" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="R3" s="22" t="s">
+      <c r="S3" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="S3" s="22" t="s">
+      <c r="T3" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="T3" s="22" t="s">
+      <c r="U3" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="W3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="X3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="Y3" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="Y3" s="2" t="s">
+      <c r="Z3" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="Z3" s="2" t="s">
+      <c r="AA3" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AA3" s="2" t="s">
+      <c r="AB3" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AB3" s="2" t="s">
+      <c r="AC3" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AC3" s="2" t="s">
+      <c r="AD3" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AD3" s="2" t="s">
+      <c r="AE3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AE3" s="2" t="s">
+      <c r="AF3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AF3" s="2" t="s">
+      <c r="AG3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AG3" s="2" t="s">
+      <c r="AH3" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>1</v>
       </c>
@@ -1497,33 +1518,35 @@
       <c r="M4" s="3">
         <v>20260105</v>
       </c>
-      <c r="N4" s="3"/>
-      <c r="O4" s="5" t="s">
+      <c r="N4" s="6">
+        <v>20260311</v>
+      </c>
+      <c r="O4" s="3"/>
+      <c r="P4" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P4" s="5">
+      <c r="Q4" s="5">
         <v>21030100</v>
       </c>
-      <c r="Q4" s="23" t="s">
+      <c r="R4" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="R4" s="23" t="s">
+      <c r="S4" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="S4" s="23" t="s">
+      <c r="T4" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="T4" s="23" t="s">
+      <c r="U4" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="U4" s="25"/>
-      <c r="V4" s="6">
+      <c r="V4" s="25"/>
+      <c r="W4" s="6">
         <v>7</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="X4" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="X4" s="5"/>
       <c r="Y4" s="5"/>
       <c r="Z4" s="5"/>
       <c r="AA4" s="5"/>
@@ -1533,8 +1556,9 @@
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
       <c r="AG4" s="5"/>
+      <c r="AH4" s="5"/>
     </row>
-    <row r="5" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -1568,52 +1592,55 @@
       <c r="M5" s="3">
         <v>20260105</v>
       </c>
-      <c r="N5" s="3"/>
-      <c r="O5" s="5" t="s">
+      <c r="N5" s="6">
+        <v>20260311</v>
+      </c>
+      <c r="O5" s="3"/>
+      <c r="P5" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="23"/>
+      <c r="Q5" s="5"/>
       <c r="R5" s="23"/>
       <c r="S5" s="23"/>
       <c r="T5" s="23"/>
-      <c r="U5" s="7"/>
-      <c r="V5" s="6">
+      <c r="U5" s="23"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="6">
         <v>7</v>
       </c>
-      <c r="W5" s="5" t="s">
+      <c r="X5" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="X5" s="5">
+      <c r="Y5" s="5">
         <v>100000</v>
       </c>
-      <c r="Y5" s="5" t="s">
+      <c r="Z5" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="Z5" s="25" t="s">
+      <c r="AA5" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="AA5" s="44">
+      <c r="AB5" s="43">
         <v>46032</v>
       </c>
-      <c r="AB5" s="5" t="s">
+      <c r="AC5" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="AC5" s="5"/>
-      <c r="AD5" s="5" t="s">
+      <c r="AD5" s="5"/>
+      <c r="AE5" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AE5" s="15" t="s">
+      <c r="AF5" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="AF5" s="5" t="s">
+      <c r="AG5" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="AG5" s="5" t="s">
+      <c r="AH5" s="5" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>1</v>
       </c>
@@ -1649,23 +1676,25 @@
       <c r="M6" s="3">
         <v>20260105</v>
       </c>
-      <c r="N6" s="3"/>
-      <c r="O6" s="5" t="s">
+      <c r="N6" s="6">
+        <v>20260311</v>
+      </c>
+      <c r="O6" s="3"/>
+      <c r="P6" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="23"/>
+      <c r="Q6" s="5"/>
       <c r="R6" s="23"/>
       <c r="S6" s="23"/>
       <c r="T6" s="23"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="6">
+      <c r="U6" s="23"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="6">
         <v>7</v>
       </c>
-      <c r="W6" s="5" t="s">
+      <c r="X6" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="X6" s="5"/>
       <c r="Y6" s="5"/>
       <c r="Z6" s="5"/>
       <c r="AA6" s="5"/>
@@ -1675,8 +1704,9 @@
       <c r="AE6" s="5"/>
       <c r="AF6" s="5"/>
       <c r="AG6" s="5"/>
+      <c r="AH6" s="5"/>
     </row>
-    <row r="7" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>2</v>
       </c>
@@ -1710,33 +1740,35 @@
       <c r="M7" s="3">
         <v>20260105</v>
       </c>
-      <c r="N7" s="3"/>
-      <c r="O7" s="5" t="s">
+      <c r="N7" s="6">
+        <v>20260312</v>
+      </c>
+      <c r="O7" s="3"/>
+      <c r="P7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P7" s="5">
+      <c r="Q7" s="5">
         <v>21030100</v>
       </c>
-      <c r="Q7" s="23" t="s">
+      <c r="R7" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="R7" s="23" t="s">
+      <c r="S7" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="S7" s="23" t="s">
+      <c r="T7" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="T7" s="23" t="s">
+      <c r="U7" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="U7" s="25"/>
-      <c r="V7" s="6">
+      <c r="V7" s="25"/>
+      <c r="W7" s="6">
         <v>7</v>
       </c>
-      <c r="W7" s="5" t="s">
+      <c r="X7" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="X7" s="5"/>
       <c r="Y7" s="5"/>
       <c r="Z7" s="5"/>
       <c r="AA7" s="5"/>
@@ -1746,8 +1778,9 @@
       <c r="AE7" s="5"/>
       <c r="AF7" s="5"/>
       <c r="AG7" s="5"/>
+      <c r="AH7" s="5"/>
     </row>
-    <row r="8" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>2</v>
       </c>
@@ -1781,52 +1814,55 @@
       <c r="M8" s="3">
         <v>20260105</v>
       </c>
-      <c r="N8" s="3"/>
-      <c r="O8" s="5" t="s">
+      <c r="N8" s="6">
+        <v>20260312</v>
+      </c>
+      <c r="O8" s="3"/>
+      <c r="P8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="23"/>
+      <c r="Q8" s="5"/>
       <c r="R8" s="23"/>
       <c r="S8" s="23"/>
       <c r="T8" s="23"/>
-      <c r="U8" s="7"/>
-      <c r="V8" s="6">
+      <c r="U8" s="23"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="6">
         <v>7</v>
       </c>
-      <c r="W8" s="5" t="s">
+      <c r="X8" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="X8" s="5">
+      <c r="Y8" s="5">
         <v>100000</v>
       </c>
-      <c r="Y8" s="5" t="s">
+      <c r="Z8" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="Z8" s="25" t="s">
+      <c r="AA8" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="AA8" s="44">
+      <c r="AB8" s="43">
         <v>46037</v>
       </c>
-      <c r="AB8" s="5" t="s">
+      <c r="AC8" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AC8" s="5"/>
-      <c r="AD8" s="5" t="s">
+      <c r="AD8" s="5"/>
+      <c r="AE8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AE8" s="5" t="s">
+      <c r="AF8" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AF8" s="5" t="s">
+      <c r="AG8" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AG8" s="5" t="s">
+      <c r="AH8" s="5" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>2</v>
       </c>
@@ -1862,23 +1898,25 @@
       <c r="M9" s="3">
         <v>20260105</v>
       </c>
-      <c r="N9" s="3"/>
-      <c r="O9" s="5" t="s">
+      <c r="N9" s="6">
+        <v>20260312</v>
+      </c>
+      <c r="O9" s="3"/>
+      <c r="P9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="23"/>
+      <c r="Q9" s="5"/>
       <c r="R9" s="23"/>
       <c r="S9" s="23"/>
       <c r="T9" s="23"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="6">
+      <c r="U9" s="23"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="6">
         <v>7</v>
       </c>
-      <c r="W9" s="5" t="s">
+      <c r="X9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="X9" s="5"/>
       <c r="Y9" s="5"/>
       <c r="Z9" s="5"/>
       <c r="AA9" s="5"/>
@@ -1888,8 +1926,9 @@
       <c r="AE9" s="5"/>
       <c r="AF9" s="5"/>
       <c r="AG9" s="5"/>
+      <c r="AH9" s="5"/>
     </row>
-    <row r="10" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>3</v>
       </c>
@@ -1923,33 +1962,35 @@
       <c r="M10" s="3">
         <v>20260105</v>
       </c>
-      <c r="N10" s="3"/>
-      <c r="O10" s="5" t="s">
+      <c r="N10" s="6">
+        <v>20260313</v>
+      </c>
+      <c r="O10" s="3"/>
+      <c r="P10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P10" s="5">
+      <c r="Q10" s="5">
         <v>21030100</v>
       </c>
-      <c r="Q10" s="23" t="s">
+      <c r="R10" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="R10" s="23" t="s">
+      <c r="S10" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="S10" s="23" t="s">
+      <c r="T10" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="T10" s="23" t="s">
+      <c r="U10" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="U10" s="25"/>
-      <c r="V10" s="6">
+      <c r="V10" s="25"/>
+      <c r="W10" s="6">
         <v>7</v>
       </c>
-      <c r="W10" s="5" t="s">
+      <c r="X10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="X10" s="5"/>
       <c r="Y10" s="5"/>
       <c r="Z10" s="5"/>
       <c r="AA10" s="5"/>
@@ -1959,8 +2000,9 @@
       <c r="AE10" s="5"/>
       <c r="AF10" s="5"/>
       <c r="AG10" s="5"/>
+      <c r="AH10" s="5"/>
     </row>
-    <row r="11" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>3</v>
       </c>
@@ -1994,52 +2036,55 @@
       <c r="M11" s="3">
         <v>20260105</v>
       </c>
-      <c r="N11" s="3"/>
-      <c r="O11" s="5" t="s">
+      <c r="N11" s="6">
+        <v>20260313</v>
+      </c>
+      <c r="O11" s="3"/>
+      <c r="P11" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="23"/>
+      <c r="Q11" s="5"/>
       <c r="R11" s="23"/>
       <c r="S11" s="23"/>
       <c r="T11" s="23"/>
-      <c r="U11" s="7"/>
-      <c r="V11" s="6">
+      <c r="U11" s="23"/>
+      <c r="V11" s="7"/>
+      <c r="W11" s="6">
         <v>7</v>
       </c>
-      <c r="W11" s="5" t="s">
+      <c r="X11" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="X11" s="5">
+      <c r="Y11" s="5">
         <v>100000</v>
       </c>
-      <c r="Y11" s="5" t="s">
+      <c r="Z11" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="Z11" s="25" t="s">
+      <c r="AA11" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="AA11" s="44">
+      <c r="AB11" s="43">
         <v>46043</v>
       </c>
-      <c r="AB11" s="5" t="s">
+      <c r="AC11" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AC11" s="5"/>
-      <c r="AD11" s="5" t="s">
+      <c r="AD11" s="5"/>
+      <c r="AE11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AE11" s="5" t="s">
+      <c r="AF11" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AF11" s="5" t="s">
+      <c r="AG11" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="AG11" s="5" t="s">
+      <c r="AH11" s="5" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="12" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>3</v>
       </c>
@@ -2075,23 +2120,25 @@
       <c r="M12" s="3">
         <v>20260105</v>
       </c>
-      <c r="N12" s="3"/>
-      <c r="O12" s="5" t="s">
+      <c r="N12" s="6">
+        <v>20260313</v>
+      </c>
+      <c r="O12" s="3"/>
+      <c r="P12" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="23"/>
+      <c r="Q12" s="5"/>
       <c r="R12" s="23"/>
       <c r="S12" s="23"/>
       <c r="T12" s="23"/>
-      <c r="U12" s="3"/>
-      <c r="V12" s="6">
+      <c r="U12" s="23"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="6">
         <v>7</v>
       </c>
-      <c r="W12" s="5" t="s">
+      <c r="X12" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="X12" s="5"/>
       <c r="Y12" s="5"/>
       <c r="Z12" s="5"/>
       <c r="AA12" s="5"/>
@@ -2101,8 +2148,9 @@
       <c r="AE12" s="5"/>
       <c r="AF12" s="5"/>
       <c r="AG12" s="5"/>
+      <c r="AH12" s="5"/>
     </row>
-    <row r="13" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>4</v>
       </c>
@@ -2136,33 +2184,35 @@
       <c r="M13" s="3">
         <v>20260105</v>
       </c>
-      <c r="N13" s="3"/>
-      <c r="O13" s="5" t="s">
+      <c r="N13" s="6">
+        <v>20260317</v>
+      </c>
+      <c r="O13" s="3"/>
+      <c r="P13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P13" s="5">
+      <c r="Q13" s="5">
         <v>21030100</v>
       </c>
-      <c r="Q13" s="23" t="s">
+      <c r="R13" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="R13" s="23" t="s">
+      <c r="S13" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="S13" s="23" t="s">
+      <c r="T13" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="T13" s="23" t="s">
+      <c r="U13" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="U13" s="25"/>
-      <c r="V13" s="6">
+      <c r="V13" s="25"/>
+      <c r="W13" s="6">
         <v>7</v>
       </c>
-      <c r="W13" s="5" t="s">
+      <c r="X13" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X13" s="5"/>
       <c r="Y13" s="5"/>
       <c r="Z13" s="5"/>
       <c r="AA13" s="5"/>
@@ -2172,8 +2222,9 @@
       <c r="AE13" s="5"/>
       <c r="AF13" s="5"/>
       <c r="AG13" s="5"/>
+      <c r="AH13" s="5"/>
     </row>
-    <row r="14" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -2207,52 +2258,55 @@
       <c r="M14" s="3">
         <v>20260105</v>
       </c>
-      <c r="N14" s="3"/>
-      <c r="O14" s="5" t="s">
+      <c r="N14" s="6">
+        <v>20260317</v>
+      </c>
+      <c r="O14" s="3"/>
+      <c r="P14" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="23"/>
+      <c r="Q14" s="5"/>
       <c r="R14" s="23"/>
       <c r="S14" s="23"/>
       <c r="T14" s="23"/>
-      <c r="U14" s="7"/>
-      <c r="V14" s="6">
+      <c r="U14" s="23"/>
+      <c r="V14" s="7"/>
+      <c r="W14" s="6">
         <v>7</v>
       </c>
-      <c r="W14" s="5" t="s">
+      <c r="X14" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X14" s="5">
+      <c r="Y14" s="5">
         <v>100000</v>
       </c>
-      <c r="Y14" s="5" t="s">
+      <c r="Z14" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="Z14" s="25" t="s">
+      <c r="AA14" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="AA14" s="44">
+      <c r="AB14" s="43">
         <v>46053</v>
       </c>
-      <c r="AB14" s="5" t="s">
+      <c r="AC14" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="AC14" s="5"/>
-      <c r="AD14" s="5" t="s">
+      <c r="AD14" s="5"/>
+      <c r="AE14" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AE14" s="5" t="s">
+      <c r="AF14" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="AF14" s="5" t="s">
+      <c r="AG14" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="AG14" s="5" t="s">
+      <c r="AH14" s="5" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:34" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>4</v>
       </c>
@@ -2288,23 +2342,25 @@
       <c r="M15" s="3">
         <v>20260105</v>
       </c>
-      <c r="N15" s="3"/>
-      <c r="O15" s="5" t="s">
+      <c r="N15" s="6">
+        <v>20260317</v>
+      </c>
+      <c r="O15" s="3"/>
+      <c r="P15" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="23"/>
+      <c r="Q15" s="5"/>
       <c r="R15" s="23"/>
       <c r="S15" s="23"/>
       <c r="T15" s="23"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="6">
+      <c r="U15" s="23"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="6">
         <v>7</v>
       </c>
-      <c r="W15" s="5" t="s">
+      <c r="X15" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X15" s="5"/>
       <c r="Y15" s="5"/>
       <c r="Z15" s="5"/>
       <c r="AA15" s="5"/>
@@ -2314,94 +2370,30 @@
       <c r="AE15" s="5"/>
       <c r="AF15" s="5"/>
       <c r="AG15" s="5"/>
+      <c r="AH15" s="5"/>
+    </row>
+    <row r="244" spans="14:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N244" s="45"/>
+    </row>
+    <row r="245" spans="14:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N245" s="45"/>
+    </row>
+    <row r="246" spans="14:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N246" s="45"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:W3" xr:uid="{8C1398C5-904C-49F7-9674-3AEBD223EAA3}"/>
+  <autoFilter ref="A3:X3" xr:uid="{8C1398C5-904C-49F7-9674-3AEBD223EAA3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ceba343f8a154e61a69d6f3ab6653fa8 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ceba343f8a154e61a69d6f3ab6653fa8>
-    <T_x00ec_nhTr_x1ea1_ngThanhTo_x00e1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Ng_x01b0__x1edd_iTr_x00ec_nh xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iTr_x00ec_nh>
-    <M_x1ee5_c_x0110__x00ed_chS_x1eed_d_x1ee5_ng xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Ng_x01b0__x1edd_iThanhTo_x00e1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iThanhTo_x00e1_n>
-    <Ng_x01b0__x1edd_iDuy_x1ec7_t40 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iDuy_x1ec7_t40>
-    <Ng_x01b0__x1edd_iCungC_x1ea5_pTh_x00f4_ngTin xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iCungC_x1ea5_pTh_x00f4_ngTin>
-    <Team xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <S_x1ed1_H_x00f3_a_x0110__x01a1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Hi_x1ec7_uL_x1ef1_c_x0110__x1ebf_nNg_x00e0_y xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Ng_x01b0__x1edd_iDuy_x1ec7_t xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iDuy_x1ec7_t>
-    <Ng_x01b0__x1edd_iDUy_x1ec7_t4 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iDUy_x1ec7_t4>
-    <_Flow_SignoffStatus xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <N_x1ed9_idung xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <S_x1ed1_Ti_x1ec1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Ng_x01b0__x1edd_iDuy_x1ec7_t2 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Ng_x01b0__x1edd_iDuy_x1ec7_t2>
-    <Th_x00e1_ngTr_x00ec_nhThanhTo_x00e1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <T_x00ea_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <TaxCatchAll xmlns="184e74be-7873-4698-965f-b07e52c33735" xsi:nil="true"/>
-    <C_x00f4_ngTy xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <_x0110__x1ed1_iT_x00e1_c_x002f_NCC xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Tags xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <DocType xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Hi_x1ec7_uL_x1ef1_cT_x1eeb_Ng_x00e0_y xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Th_x1edd_iH_x1ea1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Nofile xmlns="021df570-2223-4e8c-a451-093e8633b3bb">false</Nofile>
-    <itemFile xmlns="021df570-2223-4e8c-a451-093e8633b3bb">true</itemFile>
-    <Ph_x00e2_nlo_x1ea1_i xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-    <Uu_Tien xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2995,27 +2987,92 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ceba343f8a154e61a69d6f3ab6653fa8 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ceba343f8a154e61a69d6f3ab6653fa8>
+    <T_x00ec_nhTr_x1ea1_ngThanhTo_x00e1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Ng_x01b0__x1edd_iTr_x00ec_nh xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iTr_x00ec_nh>
+    <M_x1ee5_c_x0110__x00ed_chS_x1eed_d_x1ee5_ng xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Ng_x01b0__x1edd_iThanhTo_x00e1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iThanhTo_x00e1_n>
+    <Ng_x01b0__x1edd_iDuy_x1ec7_t40 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iDuy_x1ec7_t40>
+    <Ng_x01b0__x1edd_iCungC_x1ea5_pTh_x00f4_ngTin xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iCungC_x1ea5_pTh_x00f4_ngTin>
+    <Team xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <S_x1ed1_H_x00f3_a_x0110__x01a1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Hi_x1ec7_uL_x1ef1_c_x0110__x1ebf_nNg_x00e0_y xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Ng_x01b0__x1edd_iDuy_x1ec7_t xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iDuy_x1ec7_t>
+    <Ng_x01b0__x1edd_iDUy_x1ec7_t4 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iDUy_x1ec7_t4>
+    <_Flow_SignoffStatus xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <N_x1ed9_idung xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <S_x1ed1_Ti_x1ec1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Ng_x01b0__x1edd_iDuy_x1ec7_t2 xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Ng_x01b0__x1edd_iDuy_x1ec7_t2>
+    <Th_x00e1_ngTr_x00ec_nhThanhTo_x00e1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="021df570-2223-4e8c-a451-093e8633b3bb">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <T_x00ea_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <TaxCatchAll xmlns="184e74be-7873-4698-965f-b07e52c33735" xsi:nil="true"/>
+    <C_x00f4_ngTy xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <_x0110__x1ed1_iT_x00e1_c_x002f_NCC xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Tags xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <DocType xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Hi_x1ec7_uL_x1ef1_cT_x1eeb_Ng_x00e0_y xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Th_x1edd_iH_x1ea1_n xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Nofile xmlns="021df570-2223-4e8c-a451-093e8633b3bb">false</Nofile>
+    <itemFile xmlns="021df570-2223-4e8c-a451-093e8633b3bb">true</itemFile>
+    <Ph_x00e2_nlo_x1ea1_i xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+    <Uu_Tien xmlns="021df570-2223-4e8c-a451-093e8633b3bb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5FC039A-10D3-4E27-8A64-0E93DD51F6ED}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03548B29-A949-45C5-969C-6A63F40A3028}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="184e74be-7873-4698-965f-b07e52c33735"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="021df570-2223-4e8c-a451-093e8633b3bb"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3040,9 +3097,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03548B29-A949-45C5-969C-6A63F40A3028}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5FC039A-10D3-4E27-8A64-0E93DD51F6ED}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="184e74be-7873-4698-965f-b07e52c33735"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="021df570-2223-4e8c-a451-093e8633b3bb"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>